<commit_message>
docs(data-dictionary): บันทึก deviation Mobile-as-entry-point ของ DeviceConfigOverride (#232)
DEVICE_CONFIG_OVERRIDE.overridden_by เดิมระบุว่า "ตัดออกจาก Mobile ถาวร" (ดีไซน์
ก่อนมติ 2026-09-24) แต่ actual implementation (issue #223, PR #225/#228/#230)
แยกเป็น 2 ขั้นตอน: ST ส่งคำขอ override (pending) ได้จาก Mobile เท่านั้น ส่วน
Operation ยังคงอนุมัติ/ปฏิเสธผ่าน Web เท่านั้นเหมือนเดิม (Separation of Duty
ไม่เปลี่ยน)

อัปเดต 3 จุดตามโครงสร้างไฟล์เดิม:
- ชีท "Data Dictionary" แถว 160 (Content column) + ตั้ง "New?" เป็น "แก้ไข"
- ชีท "By Table" แถว 237 (มิเรอร์เนื้อหาเดียวกัน)
- ชีท "Overview" เพิ่ม changelog "ปรับปรุงรอบ 6" ต่อจากรอบ 1-5 เดิม
</commit_message>
<xml_diff>
--- a/docs/database/GPS_Data_Dictionary.xlsx
+++ b/docs/database/GPS_Data_Dictionary.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="5" customWidth="1" style="22" min="1" max="1"/>
@@ -853,6 +853,13 @@
       <c r="A25" t="inlineStr">
         <is>
           <t>ปรับปรุงรอบ 5 (2026-09-22, kittiphong, issue #115): เพิ่มตาราง TASK เข้ากลุ่ม “User Access &amp; Audit” — implement จริงในระบบตั้งแต่ PR #72 (Mobile Task Management) แต่ไม่เคยอยู่ใน dictionary นี้เลย field ทั้งหมดตรงกับ backend/prisma/schema.prisma model Task ปัจจุบัน (ไม่ใช่สเปกเก่าที่ตกยุค) config_id/campaign_id อ้างอิง model Config/Campaign จริง — คนละตารางกับ CONFIG_TEMPLATE/DEPLOYMENT_CAMPAIGN ที่มีอยู่แล้วในชีทนี้ (design เดิมจาก PDF ที่ยังไม่ reconcile กับของจริง นอกขอบเขตของ issue นี้ บันทึกไว้ในคอลัมน์ Content ของแต่ละ field ด้วย) · ไม่แก้ชีท “Relationships (ERD)” รอบนี้ (ตามแบบเดียวกับตอนเพิ่ม NOTIFICATION ก่อนหน้าที่ก็ไม่เคยถูกเพิ่มเข้า ERD เช่นกัน)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ปรับปรุงรอบ 6 (2026-09-29, kittiphong, issue #232): บันทึก deviation ใน DEVICE_CONFIG_OVERRIDE.overridden_by (ชีท "Data Dictionary" แถว 160 และ "By Table" แถว 237) ว่า Mobile เป็น entry point สำหรับ ST ส่งคำขอ Override (pending) ได้จริงตั้งแต่ issue #223 — ต่างจากดีไซน์เดิมในไฟล์นี้ที่ระบุว่า "ตัดออกจาก Mobile ถาวร" · Operation ยังคงเป็นผู้อนุมัติ/ปฏิเสธผ่าน Web เท่านั้น (Separation of Duty ไม่เปลี่ยน) — อ้างอิง PR #225, #228, #230</t>
         </is>
       </c>
     </row>
@@ -6976,10 +6983,14 @@
       </c>
       <c r="H160" s="6" t="inlineStr">
         <is>
-          <t>ผู้ทำการ Override (Role Operation, Senior Technician หรือ Operation - Technician) — ดำเนินการผ่านหน้าจอ Device Config Override บน Web เท่านั้น (ตัดออกจาก Mobile ถาวรตามคำสั่งหัวหน้าโปรเจกต์)</t>
-        </is>
-      </c>
-      <c r="I160" s="23" t="n"/>
+          <t>ผู้ทำการ Override (Role Operation, Senior Technician หรือ Operation - Technician) — ดำเนินการผ่านหน้าจอ Device Config Override บน Web เท่านั้น (ตัดออกจาก Mobile ถาวรตามคำสั่งหัวหน้าโปรเจกต์) — **Deviation บันทึกเพิ่ม (2026-09-29, kittiphong, issue #232, อ้างอิง #223 [ปิดแล้ว] / PR #225, #228, #230):** ข้อความข้างต้น ("ตัดออกจาก Mobile ถาวร") เป็นมติเดิมที่ถูกเปลี่ยนภายหลัง — ปัจจุบันแยกเป็น 2 ขั้นตอน: **ส่งคำขอ** ทำได้จาก Mobile โดย ST เท่านั้น (POST /devices/{deviceId}/config-override, สถานะเริ่มต้น pending) ส่วน **อนุมัติ/ปฏิเสธ** ยังคงทำได้จาก Web โดย Operation เท่านั้นเหมือนเดิม (Separation of Duty ไม่เปลี่ยน) — field overridden_by นี้จึงหมายถึงผู้ส่งคำขอ (ST ผ่าน Mobile) ไม่ใช่ผู้ตัดสินใจอีกต่อไป</t>
+        </is>
+      </c>
+      <c r="I160" s="23" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
+        </is>
+      </c>
     </row>
     <row r="161" ht="27.6" customHeight="1" s="22">
       <c r="A161" s="23" t="inlineStr">
@@ -19945,7 +19956,7 @@
       </c>
       <c r="F237" s="6" t="inlineStr">
         <is>
-          <t>ผู้ทำการ Override (Role Operation, Senior Technician หรือ Operation - Technician) — ดำเนินการผ่านหน้าจอ Device Config Override บน Web เท่านั้น (ตัดออกจาก Mobile ถาวรตามคำสั่งหัวหน้าโปรเจกต์)</t>
+          <t>ผู้ทำการ Override (Role Operation, Senior Technician หรือ Operation - Technician) — ดำเนินการผ่านหน้าจอ Device Config Override บน Web เท่านั้น (ตัดออกจาก Mobile ถาวรตามคำสั่งหัวหน้าโปรเจกต์) — **Deviation บันทึกเพิ่ม (2026-09-29, kittiphong, issue #232, อ้างอิง #223 [ปิดแล้ว] / PR #225, #228, #230):** ข้อความข้างต้น ("ตัดออกจาก Mobile ถาวร") เป็นมติเดิมที่ถูกเปลี่ยนภายหลัง — ปัจจุบันแยกเป็น 2 ขั้นตอน: **ส่งคำขอ** ทำได้จาก Mobile โดย ST เท่านั้น (POST /devices/{deviceId}/config-override, สถานะเริ่มต้น pending) ส่วน **อนุมัติ/ปฏิเสธ** ยังคงทำได้จาก Web โดย Operation เท่านั้นเหมือนเดิม (Separation of Duty ไม่เปลี่ยน) — field overridden_by นี้จึงหมายถึงผู้ส่งคำขอ (ST ผ่าน Mobile) ไม่ใช่ผู้ตัดสินใจอีกต่อไป</t>
         </is>
       </c>
     </row>
@@ -26134,63 +26145,63 @@
     </row>
   </sheetData>
   <mergeCells count="58">
+    <mergeCell ref="A316:F316"/>
+    <mergeCell ref="A448:F448"/>
+    <mergeCell ref="A292:F292"/>
     <mergeCell ref="A268:F268"/>
+    <mergeCell ref="A255:F255"/>
     <mergeCell ref="A164:F164"/>
+    <mergeCell ref="A326:F326"/>
     <mergeCell ref="A189:F189"/>
     <mergeCell ref="A394:F394"/>
     <mergeCell ref="A522:F522"/>
+    <mergeCell ref="A438:F438"/>
+    <mergeCell ref="A365:F365"/>
+    <mergeCell ref="A456:F456"/>
+    <mergeCell ref="A285:F285"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="A86:F86"/>
+    <mergeCell ref="A104:F104"/>
     <mergeCell ref="A239:F239"/>
+    <mergeCell ref="A113:F113"/>
     <mergeCell ref="A71:F71"/>
+    <mergeCell ref="A468:F468"/>
     <mergeCell ref="A307:F307"/>
+    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A203:F203"/>
+    <mergeCell ref="A489:F489"/>
     <mergeCell ref="A144:F144"/>
+    <mergeCell ref="A254:F254"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A373:F373"/>
     <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A373:F373"/>
+    <mergeCell ref="A504:F504"/>
+    <mergeCell ref="A122:F122"/>
+    <mergeCell ref="A184:F184"/>
     <mergeCell ref="A134:F134"/>
+    <mergeCell ref="A513:F513"/>
+    <mergeCell ref="A327:F327"/>
     <mergeCell ref="A152:F152"/>
     <mergeCell ref="A416:F416"/>
+    <mergeCell ref="A65:F65"/>
     <mergeCell ref="A93:F93"/>
+    <mergeCell ref="A382:F382"/>
     <mergeCell ref="A229:F229"/>
+    <mergeCell ref="A211:F211"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="A353:F353"/>
+    <mergeCell ref="A220:F220"/>
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="A143:F143"/>
+    <mergeCell ref="A403:F403"/>
     <mergeCell ref="A455:F455"/>
     <mergeCell ref="A64:F64"/>
     <mergeCell ref="A402:F402"/>
     <mergeCell ref="A300:F300"/>
+    <mergeCell ref="A488:F488"/>
     <mergeCell ref="A78:F78"/>
     <mergeCell ref="A498:F498"/>
-    <mergeCell ref="A65:F65"/>
-    <mergeCell ref="A316:F316"/>
-    <mergeCell ref="A448:F448"/>
-    <mergeCell ref="A292:F292"/>
-    <mergeCell ref="A255:F255"/>
-    <mergeCell ref="A326:F326"/>
-    <mergeCell ref="A438:F438"/>
-    <mergeCell ref="A365:F365"/>
-    <mergeCell ref="A456:F456"/>
-    <mergeCell ref="A285:F285"/>
-    <mergeCell ref="A104:F104"/>
-    <mergeCell ref="A113:F113"/>
-    <mergeCell ref="A468:F468"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A489:F489"/>
-    <mergeCell ref="A254:F254"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A504:F504"/>
-    <mergeCell ref="A122:F122"/>
-    <mergeCell ref="A184:F184"/>
-    <mergeCell ref="A513:F513"/>
-    <mergeCell ref="A327:F327"/>
-    <mergeCell ref="A382:F382"/>
-    <mergeCell ref="A211:F211"/>
-    <mergeCell ref="A220:F220"/>
-    <mergeCell ref="A403:F403"/>
-    <mergeCell ref="A488:F488"/>
     <mergeCell ref="A196:F196"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(data-dictionary): บันทึก deviation Mobile-as-entry-point ของ DeviceConfigOverride (#232) (#237)
DEVICE_CONFIG_OVERRIDE.overridden_by เดิมระบุว่า "ตัดออกจาก Mobile ถาวร" (ดีไซน์
ก่อนมติ 2026-09-24) แต่ actual implementation (issue #223, PR #225/#228/#230)
แยกเป็น 2 ขั้นตอน: ST ส่งคำขอ override (pending) ได้จาก Mobile เท่านั้น ส่วน
Operation ยังคงอนุมัติ/ปฏิเสธผ่าน Web เท่านั้นเหมือนเดิม (Separation of Duty
ไม่เปลี่ยน)

อัปเดต 3 จุดตามโครงสร้างไฟล์เดิม:
- ชีท "Data Dictionary" แถว 160 (Content column) + ตั้ง "New?" เป็น "แก้ไข"
- ชีท "By Table" แถว 237 (มิเรอร์เนื้อหาเดียวกัน)
- ชีท "Overview" เพิ่ม changelog "ปรับปรุงรอบ 6" ต่อจากรอบ 1-5 เดิม

Co-authored-by: kittiphongkubkub <kittiphongkubkub@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/database/GPS_Data_Dictionary.xlsx
+++ b/docs/database/GPS_Data_Dictionary.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="5" customWidth="1" style="22" min="1" max="1"/>
@@ -853,6 +853,13 @@
       <c r="A25" t="inlineStr">
         <is>
           <t>ปรับปรุงรอบ 5 (2026-09-22, kittiphong, issue #115): เพิ่มตาราง TASK เข้ากลุ่ม “User Access &amp; Audit” — implement จริงในระบบตั้งแต่ PR #72 (Mobile Task Management) แต่ไม่เคยอยู่ใน dictionary นี้เลย field ทั้งหมดตรงกับ backend/prisma/schema.prisma model Task ปัจจุบัน (ไม่ใช่สเปกเก่าที่ตกยุค) config_id/campaign_id อ้างอิง model Config/Campaign จริง — คนละตารางกับ CONFIG_TEMPLATE/DEPLOYMENT_CAMPAIGN ที่มีอยู่แล้วในชีทนี้ (design เดิมจาก PDF ที่ยังไม่ reconcile กับของจริง นอกขอบเขตของ issue นี้ บันทึกไว้ในคอลัมน์ Content ของแต่ละ field ด้วย) · ไม่แก้ชีท “Relationships (ERD)” รอบนี้ (ตามแบบเดียวกับตอนเพิ่ม NOTIFICATION ก่อนหน้าที่ก็ไม่เคยถูกเพิ่มเข้า ERD เช่นกัน)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ปรับปรุงรอบ 6 (2026-09-29, kittiphong, issue #232): บันทึก deviation ใน DEVICE_CONFIG_OVERRIDE.overridden_by (ชีท "Data Dictionary" แถว 160 และ "By Table" แถว 237) ว่า Mobile เป็น entry point สำหรับ ST ส่งคำขอ Override (pending) ได้จริงตั้งแต่ issue #223 — ต่างจากดีไซน์เดิมในไฟล์นี้ที่ระบุว่า "ตัดออกจาก Mobile ถาวร" · Operation ยังคงเป็นผู้อนุมัติ/ปฏิเสธผ่าน Web เท่านั้น (Separation of Duty ไม่เปลี่ยน) — อ้างอิง PR #225, #228, #230</t>
         </is>
       </c>
     </row>
@@ -6976,10 +6983,14 @@
       </c>
       <c r="H160" s="6" t="inlineStr">
         <is>
-          <t>ผู้ทำการ Override (Role Operation, Senior Technician หรือ Operation - Technician) — ดำเนินการผ่านหน้าจอ Device Config Override บน Web เท่านั้น (ตัดออกจาก Mobile ถาวรตามคำสั่งหัวหน้าโปรเจกต์)</t>
-        </is>
-      </c>
-      <c r="I160" s="23" t="n"/>
+          <t>ผู้ทำการ Override (Role Operation, Senior Technician หรือ Operation - Technician) — ดำเนินการผ่านหน้าจอ Device Config Override บน Web เท่านั้น (ตัดออกจาก Mobile ถาวรตามคำสั่งหัวหน้าโปรเจกต์) — **Deviation บันทึกเพิ่ม (2026-09-29, kittiphong, issue #232, อ้างอิง #223 [ปิดแล้ว] / PR #225, #228, #230):** ข้อความข้างต้น ("ตัดออกจาก Mobile ถาวร") เป็นมติเดิมที่ถูกเปลี่ยนภายหลัง — ปัจจุบันแยกเป็น 2 ขั้นตอน: **ส่งคำขอ** ทำได้จาก Mobile โดย ST เท่านั้น (POST /devices/{deviceId}/config-override, สถานะเริ่มต้น pending) ส่วน **อนุมัติ/ปฏิเสธ** ยังคงทำได้จาก Web โดย Operation เท่านั้นเหมือนเดิม (Separation of Duty ไม่เปลี่ยน) — field overridden_by นี้จึงหมายถึงผู้ส่งคำขอ (ST ผ่าน Mobile) ไม่ใช่ผู้ตัดสินใจอีกต่อไป</t>
+        </is>
+      </c>
+      <c r="I160" s="23" t="inlineStr">
+        <is>
+          <t>แก้ไข</t>
+        </is>
+      </c>
     </row>
     <row r="161" ht="27.6" customHeight="1" s="22">
       <c r="A161" s="23" t="inlineStr">
@@ -19945,7 +19956,7 @@
       </c>
       <c r="F237" s="6" t="inlineStr">
         <is>
-          <t>ผู้ทำการ Override (Role Operation, Senior Technician หรือ Operation - Technician) — ดำเนินการผ่านหน้าจอ Device Config Override บน Web เท่านั้น (ตัดออกจาก Mobile ถาวรตามคำสั่งหัวหน้าโปรเจกต์)</t>
+          <t>ผู้ทำการ Override (Role Operation, Senior Technician หรือ Operation - Technician) — ดำเนินการผ่านหน้าจอ Device Config Override บน Web เท่านั้น (ตัดออกจาก Mobile ถาวรตามคำสั่งหัวหน้าโปรเจกต์) — **Deviation บันทึกเพิ่ม (2026-09-29, kittiphong, issue #232, อ้างอิง #223 [ปิดแล้ว] / PR #225, #228, #230):** ข้อความข้างต้น ("ตัดออกจาก Mobile ถาวร") เป็นมติเดิมที่ถูกเปลี่ยนภายหลัง — ปัจจุบันแยกเป็น 2 ขั้นตอน: **ส่งคำขอ** ทำได้จาก Mobile โดย ST เท่านั้น (POST /devices/{deviceId}/config-override, สถานะเริ่มต้น pending) ส่วน **อนุมัติ/ปฏิเสธ** ยังคงทำได้จาก Web โดย Operation เท่านั้นเหมือนเดิม (Separation of Duty ไม่เปลี่ยน) — field overridden_by นี้จึงหมายถึงผู้ส่งคำขอ (ST ผ่าน Mobile) ไม่ใช่ผู้ตัดสินใจอีกต่อไป</t>
         </is>
       </c>
     </row>
@@ -26134,63 +26145,63 @@
     </row>
   </sheetData>
   <mergeCells count="58">
+    <mergeCell ref="A316:F316"/>
+    <mergeCell ref="A448:F448"/>
+    <mergeCell ref="A292:F292"/>
     <mergeCell ref="A268:F268"/>
+    <mergeCell ref="A255:F255"/>
     <mergeCell ref="A164:F164"/>
+    <mergeCell ref="A326:F326"/>
     <mergeCell ref="A189:F189"/>
     <mergeCell ref="A394:F394"/>
     <mergeCell ref="A522:F522"/>
+    <mergeCell ref="A438:F438"/>
+    <mergeCell ref="A365:F365"/>
+    <mergeCell ref="A456:F456"/>
+    <mergeCell ref="A285:F285"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A26:F26"/>
     <mergeCell ref="A86:F86"/>
+    <mergeCell ref="A104:F104"/>
     <mergeCell ref="A239:F239"/>
+    <mergeCell ref="A113:F113"/>
     <mergeCell ref="A71:F71"/>
+    <mergeCell ref="A468:F468"/>
     <mergeCell ref="A307:F307"/>
+    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A203:F203"/>
+    <mergeCell ref="A489:F489"/>
     <mergeCell ref="A144:F144"/>
+    <mergeCell ref="A254:F254"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A373:F373"/>
     <mergeCell ref="A20:F20"/>
-    <mergeCell ref="A373:F373"/>
+    <mergeCell ref="A504:F504"/>
+    <mergeCell ref="A122:F122"/>
+    <mergeCell ref="A184:F184"/>
     <mergeCell ref="A134:F134"/>
+    <mergeCell ref="A513:F513"/>
+    <mergeCell ref="A327:F327"/>
     <mergeCell ref="A152:F152"/>
     <mergeCell ref="A416:F416"/>
+    <mergeCell ref="A65:F65"/>
     <mergeCell ref="A93:F93"/>
+    <mergeCell ref="A382:F382"/>
     <mergeCell ref="A229:F229"/>
+    <mergeCell ref="A211:F211"/>
     <mergeCell ref="A31:F31"/>
     <mergeCell ref="A353:F353"/>
+    <mergeCell ref="A220:F220"/>
     <mergeCell ref="A40:F40"/>
     <mergeCell ref="A143:F143"/>
+    <mergeCell ref="A403:F403"/>
     <mergeCell ref="A455:F455"/>
     <mergeCell ref="A64:F64"/>
     <mergeCell ref="A402:F402"/>
     <mergeCell ref="A300:F300"/>
+    <mergeCell ref="A488:F488"/>
     <mergeCell ref="A78:F78"/>
     <mergeCell ref="A498:F498"/>
-    <mergeCell ref="A65:F65"/>
-    <mergeCell ref="A316:F316"/>
-    <mergeCell ref="A448:F448"/>
-    <mergeCell ref="A292:F292"/>
-    <mergeCell ref="A255:F255"/>
-    <mergeCell ref="A326:F326"/>
-    <mergeCell ref="A438:F438"/>
-    <mergeCell ref="A365:F365"/>
-    <mergeCell ref="A456:F456"/>
-    <mergeCell ref="A285:F285"/>
-    <mergeCell ref="A104:F104"/>
-    <mergeCell ref="A113:F113"/>
-    <mergeCell ref="A468:F468"/>
-    <mergeCell ref="A14:F14"/>
-    <mergeCell ref="A489:F489"/>
-    <mergeCell ref="A254:F254"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A504:F504"/>
-    <mergeCell ref="A122:F122"/>
-    <mergeCell ref="A184:F184"/>
-    <mergeCell ref="A513:F513"/>
-    <mergeCell ref="A327:F327"/>
-    <mergeCell ref="A382:F382"/>
-    <mergeCell ref="A211:F211"/>
-    <mergeCell ref="A220:F220"/>
-    <mergeCell ref="A403:F403"/>
-    <mergeCell ref="A488:F488"/>
     <mergeCell ref="A196:F196"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>